<commit_message>
Audit the full student journey and protect saved assessment progress
</commit_message>
<xml_diff>
--- a/assets/lessons/excel-formula-fluency/sprint/datasets/L8-A5.xlsx
+++ b/assets/lessons/excel-formula-fluency/sprint/datasets/L8-A5.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="1" r:id="R8698d4f5b6f94f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R79e726d069f44162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="R59a95b24ad3b4947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys" sheetId="4" r:id="R2bda1265ffe0465e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="5" r:id="Rb621618f8ab04886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="1" r:id="Rc51182a25ccf4379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R560532b4a3c44907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="R977bc9708b9140ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys" sheetId="4" r:id="R1f5b38df6ab14ba4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="5" r:id="Ra641fe7f2d4b40cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2535,7 +2535,7 @@
         <x:v>How to submit</x:v>
       </x:c>
       <x:c r="B3" s="23" t="str">
-        <x:v>Solve in current Microsoft 365 Excel. Answers cells are intentionally empty. Any equivalent Excel formula is accepted. Paste each requested output with its formula into the lesson. Preserve leading-zero identifiers as text. All four required tasks must pass before model solutions unlock.</x:v>
+        <x:v>Solve in current Microsoft 365 Excel. Answers cells are intentionally empty. Any equivalent formula is accepted. Submit each complete output with its formula. Preserve leading-zero identifiers as text. All four required tasks unlock models. Formula examples use commas; use semicolon argument separators if your locale requires them. Keep spill ranges empty and enter their anchor formulas outside Excel Table bodies.</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -6887,7 +6887,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R065aeb37a6e9467a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62ca4c2619db426d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8958,7 +8958,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7249c19a3d104359"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re75c7716ef574eb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>